<commit_message>
Expand the technology section to nine components
Adds the bumper sensor, omni wheel, and rain sensor, and merges adjustable
cutting height into the cutting disc entry. NetRTK now points at the tail
antenna the top view shows marked "do not cover".

Every entry carries a source comment. LiDAR range, the obstacle-recognition
figures, and the omni wheel's position on the diagram remain flagged as
unconfirmed in the file header.

Zoom out six technology hotspots

LiDAR, cameras, NetRTK, bumper, rain sensor, and blades were magnified far
enough that the surrounding robot dropped out of frame, leaving no sense of
where each part sits.
</commit_message>
<xml_diff>
--- a/docs/legal-pages-information.xlsx
+++ b/docs/legal-pages-information.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD984AB-C305-4619-8918-832D7D403E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F620FFAE-F448-4C00-99F8-7B74758FC67A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="98">
   <si>
     <t>FindMyRobo — information needed to write the legal pages</t>
   </si>
@@ -288,13 +288,34 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>Within 45 days of receiving the returned item</t>
+  </si>
+  <si>
+    <t>Intallation and demo services</t>
+  </si>
+  <si>
+    <t>1 year</t>
+  </si>
+  <si>
+    <t>3-7 business days</t>
+  </si>
+  <si>
+    <t>Warranty repair</t>
+  </si>
+  <si>
+    <t>Phone call after the installation is requested on the website.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contact </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -341,6 +362,12 @@
       <sz val="9"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -406,7 +433,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -429,6 +456,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -436,8 +466,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -790,34 +820,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
     </row>
     <row r="3" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
     </row>
     <row r="5" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
@@ -892,7 +922,7 @@
       <c r="D8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="11">
+      <c r="E8" s="8">
         <v>125563010022</v>
       </c>
       <c r="F8" s="7" t="s">
@@ -912,7 +942,7 @@
       <c r="D9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="11">
+      <c r="E9" s="8">
         <v>125563010022</v>
       </c>
       <c r="F9" s="7" t="s">
@@ -973,7 +1003,7 @@
         <v>25</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>26</v>
@@ -993,7 +1023,7 @@
         <v>11</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>11</v>
+        <v>93</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>29</v>
@@ -1013,7 +1043,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>11</v>
+        <v>89</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>31</v>
@@ -1073,7 +1103,7 @@
         <v>11</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>11</v>
+        <v>94</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>38</v>
@@ -1092,9 +1122,7 @@
       <c r="D18" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E18" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E18" s="6"/>
       <c r="F18" s="7" t="s">
         <v>40</v>
       </c>
@@ -1112,7 +1140,9 @@
       <c r="D19" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E19" s="6"/>
+      <c r="E19" s="6" t="s">
+        <v>96</v>
+      </c>
       <c r="F19" s="7" t="s">
         <v>42</v>
       </c>
@@ -1131,7 +1161,7 @@
         <v>11</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>11</v>
+        <v>97</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>44</v>
@@ -1170,8 +1200,8 @@
       <c r="D22" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E22" s="6">
-        <v>5</v>
+      <c r="E22" s="12" t="s">
+        <v>49</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>50</v>
@@ -1211,7 +1241,7 @@
         <v>55</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>11</v>
+        <v>55</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>56</v>
@@ -1231,7 +1261,7 @@
         <v>59</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>11</v>
+        <v>90</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>60</v>
@@ -1251,7 +1281,7 @@
         <v>62</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>63</v>
@@ -1290,7 +1320,9 @@
       <c r="D28" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="E28" s="6"/>
+      <c r="E28" s="6" t="s">
+        <v>67</v>
+      </c>
       <c r="F28" s="7" t="s">
         <v>11</v>
       </c>
@@ -1309,7 +1341,7 @@
         <v>70</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>71</v>
@@ -1329,7 +1361,7 @@
         <v>73</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>11</v>
+        <v>73</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>11</v>
@@ -1349,7 +1381,7 @@
         <v>75</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>11</v>
+        <v>75</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>76</v>
@@ -1369,7 +1401,7 @@
         <v>78</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>11</v>
@@ -1389,7 +1421,7 @@
         <v>80</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>11</v>
+        <v>92</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>11</v>
@@ -1409,7 +1441,7 @@
         <v>82</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>11</v>
+        <v>91</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>11</v>
@@ -1429,7 +1461,7 @@
         <v>84</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>11</v>
@@ -1449,7 +1481,7 @@
         <v>86</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>11</v>
@@ -1462,6 +1494,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
   </mergeCells>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>

</xml_diff>